<commit_message>
Republish Penrith_2025_WCH: Kayak Cross individual (Time Trials) RANK from official classification (121 cells; maintainer 2026-10-21)
</commit_message>
<xml_diff>
--- a/events/Penrith_2025_WCH/Penrith_2025_WCH_start.xlsx
+++ b/events/Penrith_2025_WCH/Penrith_2025_WCH_start.xlsx
@@ -847,6 +847,11 @@
       <c r="K6" t="n">
         <v>5</v>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>NG Wee Meng</t>
@@ -910,6 +915,11 @@
       <c r="K7" t="n">
         <v>6</v>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
       <c r="R7" t="inlineStr">
         <is>
           <t>LIAO Li-Hong</t>
@@ -1162,6 +1172,11 @@
       <c r="K11" t="n">
         <v>10</v>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R11" t="inlineStr">
         <is>
           <t>LYU Luhui</t>
@@ -1225,6 +1240,11 @@
       <c r="K12" t="n">
         <v>11</v>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="R12" t="inlineStr">
         <is>
           <t>WU Shao-Hsuan</t>
@@ -1288,6 +1308,11 @@
       <c r="K13" t="n">
         <v>12</v>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="R13" t="inlineStr">
         <is>
           <t>GUBENKO Nikita</t>
@@ -1351,6 +1376,11 @@
       <c r="K14" t="n">
         <v>13</v>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
       <c r="R14" t="inlineStr">
         <is>
           <t>SMIRNOV Egor</t>
@@ -1414,6 +1444,11 @@
       <c r="K15" t="n">
         <v>14</v>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
       <c r="R15" t="inlineStr">
         <is>
           <t>SNOOK George</t>
@@ -1477,6 +1512,11 @@
       <c r="K16" t="n">
         <v>15</v>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
       <c r="R16" t="inlineStr">
         <is>
           <t>NIJHAWAN Nikhil</t>
@@ -1540,6 +1580,11 @@
       <c r="K17" t="n">
         <v>16</v>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R17" t="inlineStr">
         <is>
           <t>ZHANG Jiahao</t>
@@ -1603,6 +1648,11 @@
       <c r="K18" t="n">
         <v>17</v>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="R18" t="inlineStr">
         <is>
           <t>GONSENICA Adam</t>
@@ -1666,6 +1716,11 @@
       <c r="K19" t="n">
         <v>18</v>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
       <c r="R19" t="inlineStr">
         <is>
           <t>PLAUDIS Martins</t>
@@ -1729,6 +1784,11 @@
       <c r="K20" t="n">
         <v>19</v>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R20" t="inlineStr">
         <is>
           <t>EIGEL Pavel</t>
@@ -1792,6 +1852,11 @@
       <c r="K21" t="n">
         <v>20</v>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R21" t="inlineStr">
         <is>
           <t>KOZLOV Ivan</t>
@@ -1855,6 +1920,11 @@
       <c r="K22" t="n">
         <v>21</v>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="R22" t="inlineStr">
         <is>
           <t>TANAKA Yuuki</t>
@@ -1918,6 +1988,11 @@
       <c r="K23" t="n">
         <v>22</v>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
       <c r="R23" t="inlineStr">
         <is>
           <t>JACOB Lucas</t>
@@ -1981,6 +2056,11 @@
       <c r="K24" t="n">
         <v>23</v>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
       <c r="R24" t="inlineStr">
         <is>
           <t>MUTO Yusuke</t>
@@ -2044,6 +2124,11 @@
       <c r="K25" t="n">
         <v>24</v>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
       <c r="R25" t="inlineStr">
         <is>
           <t>REINOSO Antonio</t>
@@ -2107,6 +2192,11 @@
       <c r="K26" t="n">
         <v>25</v>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="R26" t="inlineStr">
         <is>
           <t>MAPELLI Guilherme</t>
@@ -2170,6 +2260,11 @@
       <c r="K27" t="n">
         <v>26</v>
       </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="R27" t="inlineStr">
         <is>
           <t>UKALOVIC Thomas</t>
@@ -2233,6 +2328,11 @@
       <c r="K28" t="n">
         <v>27</v>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R28" t="inlineStr">
         <is>
           <t>SOVKO Serhii</t>
@@ -2296,6 +2396,11 @@
       <c r="K29" t="n">
         <v>28</v>
       </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R29" t="inlineStr">
         <is>
           <t>BRZEZINSKI Jakub</t>
@@ -2359,6 +2464,11 @@
       <c r="K30" t="n">
         <v>29</v>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
       <c r="R30" t="inlineStr">
         <is>
           <t>CUNHA Joao</t>
@@ -2422,6 +2532,11 @@
       <c r="K31" t="n">
         <v>30</v>
       </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="R31" t="inlineStr">
         <is>
           <t>KREMSLEHNER Moritz</t>
@@ -2485,6 +2600,11 @@
       <c r="K32" t="n">
         <v>31</v>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="R32" t="inlineStr">
         <is>
           <t>BOYD Trevor</t>
@@ -2548,6 +2668,11 @@
       <c r="K33" t="n">
         <v>32</v>
       </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
       <c r="R33" t="inlineStr">
         <is>
           <t>FRIEDENSON Kaelin</t>
@@ -2611,6 +2736,11 @@
       <c r="K34" t="n">
         <v>33</v>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
       <c r="R34" t="inlineStr">
         <is>
           <t>TRIPANO Manuel</t>
@@ -2674,6 +2804,11 @@
       <c r="K35" t="n">
         <v>34</v>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
       <c r="R35" t="inlineStr">
         <is>
           <t>LOCNIKAR Jan</t>
@@ -2737,6 +2872,11 @@
       <c r="K36" t="n">
         <v>35</v>
       </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R36" t="inlineStr">
         <is>
           <t>LEITNER Mario</t>
@@ -2800,6 +2940,11 @@
       <c r="K37" t="n">
         <v>36</v>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="R37" t="inlineStr">
         <is>
           <t>ZIELONKA Mark</t>
@@ -2863,6 +3008,11 @@
       <c r="K38" t="n">
         <v>37</v>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="R38" t="inlineStr">
         <is>
           <t>ECHANIZ Pau</t>
@@ -2926,6 +3076,11 @@
       <c r="K39" t="n">
         <v>38</v>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R39" t="inlineStr">
         <is>
           <t>MCCREERY Alistair</t>
@@ -2989,6 +3144,11 @@
       <c r="K40" t="n">
         <v>39</v>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="R40" t="inlineStr">
         <is>
           <t>HUANG Liman</t>
@@ -3052,6 +3212,11 @@
       <c r="K41" t="n">
         <v>40</v>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R41" t="inlineStr">
         <is>
           <t>RUDORFER Martin</t>
@@ -3115,6 +3280,11 @@
       <c r="K42" t="n">
         <v>41</v>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R42" t="inlineStr">
         <is>
           <t>GRIGAR Jakub</t>
@@ -3178,6 +3348,11 @@
       <c r="K43" t="n">
         <v>42</v>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
       <c r="R43" t="inlineStr">
         <is>
           <t>LONG Kyler James</t>
@@ -3241,6 +3416,11 @@
       <c r="K44" t="n">
         <v>43</v>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="R44" t="inlineStr">
         <is>
           <t>ALVARENGA Frederico</t>
@@ -3304,6 +3484,11 @@
       <c r="K45" t="n">
         <v>44</v>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R45" t="inlineStr">
         <is>
           <t>HALCIN Martin</t>
@@ -3367,6 +3552,11 @@
       <c r="K46" t="n">
         <v>45</v>
       </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R46" t="inlineStr">
         <is>
           <t>FERRAZZI Xabier</t>
@@ -3430,6 +3620,11 @@
       <c r="K47" t="n">
         <v>46</v>
       </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R47" t="inlineStr">
         <is>
           <t>IVCHENKO Artem</t>
@@ -3493,6 +3688,11 @@
       <c r="K48" t="n">
         <v>47</v>
       </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R48" t="inlineStr">
         <is>
           <t>COLLIER Nicholas</t>
@@ -3556,6 +3756,11 @@
       <c r="K49" t="n">
         <v>48</v>
       </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
       <c r="R49" t="inlineStr">
         <is>
           <t>DESNOS Mathieu</t>
@@ -3619,6 +3824,11 @@
       <c r="K50" t="n">
         <v>49</v>
       </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R50" t="inlineStr">
         <is>
           <t>AUBERTIN Maxime</t>
@@ -3682,6 +3892,11 @@
       <c r="K51" t="n">
         <v>50</v>
       </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R51" t="inlineStr">
         <is>
           <t>CASTRYCK Titouan</t>
@@ -3745,6 +3960,11 @@
       <c r="K52" t="n">
         <v>51</v>
       </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R52" t="inlineStr">
         <is>
           <t>POPE Benjamin</t>
@@ -3808,6 +4028,11 @@
       <c r="K53" t="n">
         <v>52</v>
       </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R53" t="inlineStr">
         <is>
           <t>ANDERSON Timothy</t>
@@ -3871,6 +4096,11 @@
       <c r="K54" t="n">
         <v>53</v>
       </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R54" t="inlineStr">
         <is>
           <t>HENGST Stefan</t>
@@ -3934,6 +4164,11 @@
       <c r="K55" t="n">
         <v>54</v>
       </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R55" t="inlineStr">
         <is>
           <t>KUCHNO Tadeusz</t>
@@ -3997,6 +4232,11 @@
       <c r="K56" t="n">
         <v>55</v>
       </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R56" t="inlineStr">
         <is>
           <t>CHIARELLO Gelindo</t>
@@ -4060,6 +4300,11 @@
       <c r="K57" t="n">
         <v>56</v>
       </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R57" t="inlineStr">
         <is>
           <t>NOVAK Matyas</t>
@@ -4123,6 +4368,11 @@
       <c r="K58" t="n">
         <v>57</v>
       </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R58" t="inlineStr">
         <is>
           <t>ROELLER Tillmann</t>
@@ -4186,6 +4436,11 @@
       <c r="K59" t="n">
         <v>58</v>
       </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R59" t="inlineStr">
         <is>
           <t>DELFOUR Lucien</t>
@@ -4249,6 +4504,11 @@
       <c r="K60" t="n">
         <v>59</v>
       </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R60" t="inlineStr">
         <is>
           <t>KREJCI Jakub</t>
@@ -4312,6 +4572,11 @@
       <c r="K61" t="n">
         <v>60</v>
       </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R61" t="inlineStr">
         <is>
           <t>DE COSTER Gabriel</t>
@@ -4375,6 +4640,11 @@
       <c r="K62" t="n">
         <v>61</v>
       </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R62" t="inlineStr">
         <is>
           <t>BALDONI Alex</t>
@@ -4438,6 +4708,11 @@
       <c r="K63" t="n">
         <v>62</v>
       </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R63" t="inlineStr">
         <is>
           <t>LEAVER Sam</t>
@@ -4501,6 +4776,11 @@
       <c r="K64" t="n">
         <v>63</v>
       </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R64" t="inlineStr">
         <is>
           <t>HOCEVAR Ziga Lin</t>
@@ -4564,6 +4844,11 @@
       <c r="K65" t="n">
         <v>64</v>
       </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R65" t="inlineStr">
         <is>
           <t>HEGGE Noah</t>
@@ -4627,6 +4912,11 @@
       <c r="K66" t="n">
         <v>65</v>
       </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R66" t="inlineStr">
         <is>
           <t>ROHRER Jan</t>
@@ -4690,6 +4980,11 @@
       <c r="K67" t="n">
         <v>66</v>
       </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R67" t="inlineStr">
         <is>
           <t>ECHEVERRIA OLGUIN Andraz</t>
@@ -4753,6 +5048,11 @@
       <c r="K68" t="n">
         <v>67</v>
       </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R68" t="inlineStr">
         <is>
           <t>DE GENNARO Giovanni</t>
@@ -4816,6 +5116,11 @@
       <c r="K69" t="n">
         <v>68</v>
       </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R69" t="inlineStr">
         <is>
           <t>GONCALVES Pedro</t>
@@ -4879,6 +5184,11 @@
       <c r="K70" t="n">
         <v>69</v>
       </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R70" t="inlineStr">
         <is>
           <t>RENIA Benjamin</t>
@@ -4942,6 +5252,11 @@
       <c r="K71" t="n">
         <v>70</v>
       </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R71" t="inlineStr">
         <is>
           <t>DICKSON Jonny</t>
@@ -5005,6 +5320,11 @@
       <c r="K72" t="n">
         <v>71</v>
       </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R72" t="inlineStr">
         <is>
           <t>MADORE Mathurin</t>
@@ -5068,6 +5388,11 @@
       <c r="K73" t="n">
         <v>72</v>
       </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R73" t="inlineStr">
         <is>
           <t>POLACZYK Mateusz</t>
@@ -5131,6 +5456,11 @@
       <c r="K74" t="n">
         <v>73</v>
       </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R74" t="inlineStr">
         <is>
           <t>OCHOA Manuel</t>
@@ -5194,6 +5524,11 @@
       <c r="K75" t="n">
         <v>74</v>
       </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R75" t="inlineStr">
         <is>
           <t>LLORENTE David</t>
@@ -5257,6 +5592,11 @@
       <c r="K76" t="n">
         <v>75</v>
       </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R76" t="inlineStr">
         <is>
           <t>DOUGOUD Martin</t>
@@ -5320,6 +5660,11 @@
       <c r="K77" t="n">
         <v>76</v>
       </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R77" t="inlineStr">
         <is>
           <t>BUTCHER Finn</t>
@@ -5383,6 +5728,11 @@
       <c r="K78" t="n">
         <v>77</v>
       </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R78" t="inlineStr">
         <is>
           <t>CLARKE Joseph</t>
@@ -5446,6 +5796,11 @@
       <c r="K79" t="n">
         <v>78</v>
       </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R79" t="inlineStr">
         <is>
           <t>SOKOLOVA Mariia</t>
@@ -5509,6 +5864,11 @@
       <c r="K80" t="n">
         <v>79</v>
       </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="R80" t="inlineStr">
         <is>
           <t>KURIA Michelle Wambui</t>
@@ -5572,6 +5932,11 @@
       <c r="K81" t="n">
         <v>80</v>
       </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="R81" t="inlineStr">
         <is>
           <t>XHEMAJLJI Blandine</t>
@@ -5635,6 +6000,11 @@
       <c r="K82" t="n">
         <v>81</v>
       </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R82" t="inlineStr">
         <is>
           <t>CHANG Chu-Han</t>
@@ -5698,6 +6068,11 @@
       <c r="K83" t="n">
         <v>82</v>
       </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R83" t="inlineStr">
         <is>
           <t>MINAZOVA Alsu</t>
@@ -5761,6 +6136,11 @@
       <c r="K84" t="n">
         <v>83</v>
       </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R84" t="inlineStr">
         <is>
           <t>KRYLOVA Kseniia</t>
@@ -5824,6 +6204,11 @@
       <c r="K85" t="n">
         <v>84</v>
       </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="R85" t="inlineStr">
         <is>
           <t>WU Ting-I</t>
@@ -5887,6 +6272,11 @@
       <c r="K86" t="n">
         <v>85</v>
       </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R86" t="inlineStr">
         <is>
           <t>MILLS Waris</t>
@@ -5950,6 +6340,11 @@
       <c r="K87" t="n">
         <v>86</v>
       </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
       <c r="R87" t="inlineStr">
         <is>
           <t>YAZAWA Aki</t>
@@ -6013,6 +6408,11 @@
       <c r="K88" t="n">
         <v>87</v>
       </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="R88" t="inlineStr">
         <is>
           <t>LUKNAROVA Emanuela</t>
@@ -6076,6 +6476,11 @@
       <c r="K89" t="n">
         <v>88</v>
       </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R89" t="inlineStr">
         <is>
           <t>PITCHER FARRELL Cleo</t>
@@ -6139,6 +6544,11 @@
       <c r="K90" t="n">
         <v>89</v>
       </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R90" t="inlineStr">
         <is>
           <t>WILLIAMS Courtney</t>
@@ -6202,6 +6612,11 @@
       <c r="K91" t="n">
         <v>90</v>
       </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R91" t="inlineStr">
         <is>
           <t>HILGERTOVA Amalie</t>
@@ -6265,6 +6680,11 @@
       <c r="K92" t="n">
         <v>91</v>
       </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R92" t="inlineStr">
         <is>
           <t>PLATA Laura</t>
@@ -6328,6 +6748,11 @@
       <c r="K93" t="n">
         <v>92</v>
       </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R93" t="inlineStr">
         <is>
           <t>REX Rosie</t>
@@ -6391,6 +6816,11 @@
       <c r="K94" t="n">
         <v>93</v>
       </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R94" t="inlineStr">
         <is>
           <t>GORA Aleksandra</t>
@@ -6454,6 +6884,11 @@
       <c r="K95" t="n">
         <v>94</v>
       </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R95" t="inlineStr">
         <is>
           <t>BRZESKA Dominika</t>
@@ -6517,6 +6952,11 @@
       <c r="K96" t="n">
         <v>95</v>
       </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R96" t="inlineStr">
         <is>
           <t>SORRIBES Laia</t>
@@ -6580,6 +7020,11 @@
       <c r="K97" t="n">
         <v>96</v>
       </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="R97" t="inlineStr">
         <is>
           <t>O'CALLAGHAN Georgia</t>
@@ -6643,6 +7088,11 @@
       <c r="K98" t="n">
         <v>97</v>
       </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R98" t="inlineStr">
         <is>
           <t>DAVIDSON Codie</t>
@@ -6706,6 +7156,11 @@
       <c r="K99" t="n">
         <v>98</v>
       </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R99" t="inlineStr">
         <is>
           <t>STANOVSKA Sona</t>
@@ -6769,6 +7224,11 @@
       <c r="K100" t="n">
         <v>99</v>
       </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R100" t="inlineStr">
         <is>
           <t>PANKOVA Zuzana</t>
@@ -6832,6 +7292,11 @@
       <c r="K101" t="n">
         <v>100</v>
       </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R101" t="inlineStr">
         <is>
           <t>ALTMAN Marcella</t>
@@ -6895,6 +7360,11 @@
       <c r="K102" t="n">
         <v>101</v>
       </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R102" t="inlineStr">
         <is>
           <t>REINOSO Sofia</t>
@@ -6958,6 +7428,11 @@
       <c r="K103" t="n">
         <v>102</v>
       </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R103" t="inlineStr">
         <is>
           <t>US Viktoriia</t>
@@ -7021,6 +7496,11 @@
       <c r="K104" t="n">
         <v>103</v>
       </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R104" t="inlineStr">
         <is>
           <t>BAYN Nele</t>
@@ -7084,6 +7564,11 @@
       <c r="K105" t="n">
         <v>104</v>
       </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R105" t="inlineStr">
         <is>
           <t>NOVAK Ajda</t>
@@ -7147,6 +7632,11 @@
       <c r="K106" t="n">
         <v>105</v>
       </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R106" t="inlineStr">
         <is>
           <t>TEUNISSEN Lena</t>
@@ -7210,6 +7700,11 @@
       <c r="K107" t="n">
         <v>106</v>
       </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R107" t="inlineStr">
         <is>
           <t>LI Shiting</t>
@@ -7273,6 +7768,11 @@
       <c r="K108" t="n">
         <v>107</v>
       </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="R108" t="inlineStr">
         <is>
           <t>SAMKOVA Olga</t>
@@ -7336,6 +7836,11 @@
       <c r="K109" t="n">
         <v>108</v>
       </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R109" t="inlineStr">
         <is>
           <t>HERZOG Andrea</t>
@@ -7399,6 +7904,11 @@
       <c r="K110" t="n">
         <v>109</v>
       </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="R110" t="inlineStr">
         <is>
           <t>HOCEVAR Eva Alina</t>
@@ -7462,6 +7972,11 @@
       <c r="K111" t="n">
         <v>110</v>
       </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R111" t="inlineStr">
         <is>
           <t>SABATTINI Chiara</t>
@@ -7525,6 +8040,11 @@
       <c r="K112" t="n">
         <v>111</v>
       </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R112" t="inlineStr">
         <is>
           <t>LEAVER Lois</t>
@@ -7588,6 +8108,11 @@
       <c r="K113" t="n">
         <v>112</v>
       </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R113" t="inlineStr">
         <is>
           <t>LAZKANO Miren</t>
@@ -7651,6 +8176,11 @@
       <c r="K114" t="n">
         <v>113</v>
       </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R114" t="inlineStr">
         <is>
           <t>SATILA Ana</t>
@@ -7714,6 +8244,11 @@
       <c r="K115" t="n">
         <v>114</v>
       </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R115" t="inlineStr">
         <is>
           <t>DORIA Monica</t>
@@ -7777,6 +8312,11 @@
       <c r="K116" t="n">
         <v>115</v>
       </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R116" t="inlineStr">
         <is>
           <t>ESTACIA NETA Omira</t>
@@ -7840,6 +8380,11 @@
       <c r="K117" t="n">
         <v>116</v>
       </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R117" t="inlineStr">
         <is>
           <t>XIE Xueting</t>
@@ -7903,6 +8448,11 @@
       <c r="K118" t="n">
         <v>117</v>
       </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R118" t="inlineStr">
         <is>
           <t>KNEBLOVA Tereza</t>
@@ -7966,6 +8516,11 @@
       <c r="K119" t="n">
         <v>118</v>
       </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R119" t="inlineStr">
         <is>
           <t>ZWOLINSKA Klaudia</t>
@@ -8029,6 +8584,11 @@
       <c r="K120" t="n">
         <v>119</v>
       </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R120" t="inlineStr">
         <is>
           <t>SETCHELL Nikita</t>
@@ -8092,6 +8652,11 @@
       <c r="K121" t="n">
         <v>120</v>
       </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R121" t="inlineStr">
         <is>
           <t>VUITTON Emma</t>
@@ -8155,6 +8720,11 @@
       <c r="K122" t="n">
         <v>121</v>
       </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R122" t="inlineStr">
         <is>
           <t>LEIBFARTH Evy</t>
@@ -8218,6 +8788,11 @@
       <c r="K123" t="n">
         <v>122</v>
       </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R123" t="inlineStr">
         <is>
           <t>FUNK Ricarda</t>
@@ -8281,6 +8856,11 @@
       <c r="K124" t="n">
         <v>123</v>
       </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R124" t="inlineStr">
         <is>
           <t>CHOURRAUT Maialen</t>
@@ -8344,6 +8924,11 @@
       <c r="K125" t="n">
         <v>124</v>
       </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R125" t="inlineStr">
         <is>
           <t>MARX Alena</t>
@@ -8407,6 +8992,11 @@
       <c r="K126" t="n">
         <v>125</v>
       </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R126" t="inlineStr">
         <is>
           <t>FOX Noemie</t>
@@ -8470,6 +9060,11 @@
       <c r="K127" t="n">
         <v>126</v>
       </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R127" t="inlineStr">
         <is>
           <t>PRIGENT Camille</t>
@@ -8533,6 +9128,11 @@
       <c r="K128" t="n">
         <v>127</v>
       </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R128" t="inlineStr">
         <is>
           <t>HUG Angele</t>
@@ -8595,6 +9195,11 @@
       </c>
       <c r="K129" t="n">
         <v>128</v>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="R129" t="inlineStr">
         <is>

</xml_diff>